<commit_message>
Add Minimax player, play script, updated experiments and results
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/resultados.xlsx
+++ b/resultados.xlsx
@@ -523,21 +523,39 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>A preencher</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr"/>
-      <c r="D2" s="2" t="inlineStr"/>
-      <c r="E2" s="2" t="inlineStr"/>
-      <c r="F2" s="2" t="inlineStr"/>
-      <c r="G2" s="3" t="inlineStr"/>
-      <c r="H2" s="3" t="inlineStr"/>
-      <c r="I2" s="4" t="inlineStr"/>
-      <c r="J2" s="4" t="inlineStr"/>
-      <c r="K2" s="4" t="inlineStr"/>
+          <t>Minimax max_depth=4; Random sem parametros</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" s="4" t="n">
+        <v>0.5666112299986708</v>
+      </c>
+      <c r="J2" s="4" t="n">
+        <v>1.110372399998596</v>
+      </c>
+      <c r="K2" s="4" t="n">
+        <v>0.3158927000040421</v>
+      </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>A preencher pelo colega depois de adicionar MinimaxAIPlayer e a heuristica.</t>
+          <t>O Minimax avalia sistematicamente a arvore de jogo ate profundidade 4 e escolhe sempre a jogada com maior valor heuristico. O aleatorio nao planeia e perde quase sempre contra qualquer agente que calcule ameacas.</t>
         </is>
       </c>
     </row>
@@ -571,13 +589,13 @@
         <v>0</v>
       </c>
       <c r="I3" s="4" t="n">
-        <v>3.633662629999958</v>
+        <v>1.647025155001029</v>
       </c>
       <c r="J3" s="4" t="n">
-        <v>8.439887099999851</v>
+        <v>4.464260200009448</v>
       </c>
       <c r="K3" s="4" t="n">
-        <v>1.846698500000002</v>
+        <v>0.8383530999999493</v>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
@@ -593,21 +611,39 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>A preencher</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr"/>
-      <c r="D4" s="2" t="inlineStr"/>
-      <c r="E4" s="2" t="inlineStr"/>
-      <c r="F4" s="2" t="inlineStr"/>
-      <c r="G4" s="3" t="inlineStr"/>
-      <c r="H4" s="3" t="inlineStr"/>
-      <c r="I4" s="4" t="inlineStr"/>
-      <c r="J4" s="4" t="inlineStr"/>
-      <c r="K4" s="4" t="inlineStr"/>
+          <t>Minimax max_depth=3; MCTS max_iterations=25</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="H4" s="3" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="I4" s="4" t="n">
+        <v>0.4889490000001387</v>
+      </c>
+      <c r="J4" s="4" t="n">
+        <v>0.7785189999995055</v>
+      </c>
+      <c r="K4" s="4" t="n">
+        <v>0.1953909000003478</v>
+      </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>A preencher em conjunto, ajustando max_depth e max_iterations para tempos semelhantes.</t>
+          <t>Parametros calibrados para tempo por jogada equivalente (~21ms). Minimax (profundidade 3) usa poda alfa-beta e heuristica posicional. MCTS (25 iteracoes) usa simulacoes aleatorias com UCB1.</t>
         </is>
       </c>
     </row>
@@ -619,21 +655,39 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>A preencher</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr"/>
-      <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="2" t="inlineStr"/>
-      <c r="F5" s="2" t="inlineStr"/>
-      <c r="G5" s="3" t="inlineStr"/>
-      <c r="H5" s="3" t="inlineStr"/>
-      <c r="I5" s="4" t="inlineStr"/>
-      <c r="J5" s="4" t="inlineStr"/>
-      <c r="K5" s="4" t="inlineStr"/>
+          <t>Minimax max_depth=4; MCTS max_iterations=100</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H5" s="3" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="I5" s="4" t="n">
+        <v>2.602179119999346</v>
+      </c>
+      <c r="J5" s="4" t="n">
+        <v>4.883838699999615</v>
+      </c>
+      <c r="K5" s="4" t="n">
+        <v>0.9841975000017555</v>
+      </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>A preencher em conjunto, usando uma segunda combinacao de parametros.</t>
+          <t>Parametros calibrados para tempo por jogada equivalente (~86ms). Minimax (profundidade 4) usa poda alfa-beta e heuristica posicional. MCTS (100 iteracoes) usa simulacoes aleatorias com UCB1.</t>
         </is>
       </c>
     </row>
@@ -645,21 +699,39 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>A preencher</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr"/>
-      <c r="D6" s="2" t="inlineStr"/>
-      <c r="E6" s="2" t="inlineStr"/>
-      <c r="F6" s="2" t="inlineStr"/>
-      <c r="G6" s="3" t="inlineStr"/>
-      <c r="H6" s="3" t="inlineStr"/>
-      <c r="I6" s="4" t="inlineStr"/>
-      <c r="J6" s="4" t="inlineStr"/>
-      <c r="K6" s="4" t="inlineStr"/>
+          <t>Minimax max_depth=5; MCTS max_iterations=430</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="H6" s="3" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="I6" s="4" t="n">
+        <v>8.802062739998656</v>
+      </c>
+      <c r="J6" s="4" t="n">
+        <v>11.52026439999463</v>
+      </c>
+      <c r="K6" s="4" t="n">
+        <v>5.211587999991025</v>
+      </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>A preencher em conjunto, usando uma terceira combinacao de parametros.</t>
+          <t>Parametros calibrados para tempo por jogada equivalente (~380ms). Minimax (profundidade 5) usa poda alfa-beta e heuristica posicional. MCTS (430 iteracoes) usa simulacoes aleatorias com UCB1.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update results with human vs AI games
</commit_message>
<xml_diff>
--- a/resultados.xlsx
+++ b/resultados.xlsx
@@ -738,26 +738,44 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Humano vs IA (Opcional)</t>
+          <t>Humano vs Minimax</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>A preencher</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr"/>
-      <c r="D7" s="2" t="inlineStr"/>
-      <c r="E7" s="2" t="inlineStr"/>
-      <c r="F7" s="2" t="inlineStr"/>
-      <c r="G7" s="3" t="inlineStr"/>
-      <c r="H7" s="3" t="inlineStr"/>
-      <c r="I7" s="4" t="inlineStr"/>
-      <c r="J7" s="4" t="inlineStr"/>
-      <c r="K7" s="4" t="inlineStr"/>
+          <t>Humano vs Minimax max_depth=4</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="I7" s="4" t="n">
+        <v>26.25672513333336</v>
+      </c>
+      <c r="J7" s="4" t="n">
+        <v>40.78145310000002</v>
+      </c>
+      <c r="K7" s="4" t="n">
+        <v>16.67157090000001</v>
+      </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>Opcional no enunciado.</t>
+          <t>Jogos manuais. Humano (Vermelho, J1) vs Minimax com poda alfa-beta (Amarelo, J2).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update human vs AI results
</commit_message>
<xml_diff>
--- a/resultados.xlsx
+++ b/resultados.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -747,13 +747,13 @@
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D7" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F7" s="2" t="n">
         <v>0</v>
@@ -765,17 +765,61 @@
         <v>1</v>
       </c>
       <c r="I7" s="4" t="n">
-        <v>26.25672513333336</v>
+        <v>31.8814026</v>
       </c>
       <c r="J7" s="4" t="n">
-        <v>40.78145310000002</v>
+        <v>31.8814026</v>
       </c>
       <c r="K7" s="4" t="n">
-        <v>16.67157090000001</v>
+        <v>31.8814026</v>
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
           <t>Jogos manuais. Humano (Vermelho, J1) vs Minimax com poda alfa-beta (Amarelo, J2).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Humano vs MCTS</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Humano vs MCTS max_iterations=500</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="I8" s="4" t="n">
+        <v>25.8599256</v>
+      </c>
+      <c r="J8" s="4" t="n">
+        <v>25.8599256</v>
+      </c>
+      <c r="K8" s="4" t="n">
+        <v>25.8599256</v>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>Jogos manuais. Humano (Vermelho, J1) vs MCTS com UCB1 (Amarelo, J2).</t>
         </is>
       </c>
     </row>

</xml_diff>